<commit_message>
Fix the three Needs Review records (#72)
All three were data faults rather than gaps in the driver map: the Sub-type did
not describe what each record's own evidence said had failed.

Bombardier / STELIA (Product / Process Clarification -> Process / WarRoom
Creation): the supplier was resolved and the WarRoom was not created, twin of the
META row. Routed To moves with it. Sandisk / EAO-37 (People -> Process / Captured
Late): its RCA calls it a reporting delay, not a coverage gap. HPE / SEC
notification (People / Process Clarification -> Process / Captured Late): a
lateness failure with a timeliness control as its remedy, and the thinnest of the
three -- flagged for revisit if closure inputs land.

Process misses go 3 to 6, Product 46 to 45, People 29 to 27; total stays 78 and
Needs Review is empty. Caches refreshed.

Gate green: validate 0 warnings, selftest 23/23, smoke 15 pages, audit 9 pages.
</commit_message>
<xml_diff>
--- a/EventWatch_Customer_Complaints_2026.xlsx
+++ b/EventWatch_Customer_Complaints_2026.xlsx
@@ -2378,13 +2378,13 @@
                 <formatCode>General</formatCode>
                 <ptCount val="3"/>
                 <pt idx="0">
-                  <v>56</v>
+                  <v>55</v>
                 </pt>
                 <pt idx="1">
-                  <v>34</v>
+                  <v>32</v>
                 </pt>
                 <pt idx="2">
-                  <v>5</v>
+                  <v>8</v>
                 </pt>
               </numCache>
             </numRef>
@@ -6123,12 +6123,12 @@
       </c>
       <c r="I24" s="33" t="inlineStr">
         <is>
-          <t>People</t>
+          <t>Process</t>
         </is>
       </c>
       <c r="J24" s="33" t="inlineStr">
         <is>
-          <t>Process Clarification</t>
+          <t>Captured Late</t>
         </is>
       </c>
       <c r="K24" s="33" t="inlineStr">
@@ -9025,12 +9025,12 @@
       </c>
       <c r="I52" s="33" t="inlineStr">
         <is>
-          <t>Product</t>
+          <t>Process</t>
         </is>
       </c>
       <c r="J52" s="33" t="inlineStr">
         <is>
-          <t>Process Clarification</t>
+          <t>WarRoom Creation</t>
         </is>
       </c>
       <c r="K52" s="33" t="inlineStr">
@@ -9084,7 +9084,7 @@
       <c r="X52" s="33" t="n"/>
       <c r="Y52" s="33" t="inlineStr">
         <is>
-          <t>Product &amp; Platform</t>
+          <t>EventWatch Ops - Nitin Rindhe</t>
         </is>
       </c>
       <c r="Z52" s="37" t="n"/>
@@ -14587,7 +14587,7 @@
       </c>
       <c r="I103" s="33" t="inlineStr">
         <is>
-          <t>People</t>
+          <t>Process</t>
         </is>
       </c>
       <c r="J103" s="33" t="inlineStr">

</xml_diff>

<commit_message>
Correct all three Needs Review records against the evidence (#73)
Bombardier / STELIA is Product / Source Coverage -- the email thread says the feed
was never received by the application, so it never entered the portal; a supplier
being listed says nothing about whether the story arrived. Sandisk / EAO-37 is
People / Review, an analyst overlooking it, with the reporting delay as the
symptom rather than the cause. HPE is Process / Process Clarification: the news
was not public and a clarification went back.

DRIVERS gains (People, Captured Late) so a future row on that pair has a label,
and root_drivers() stops folding a single driver into Other.

Product 46, People 28, Process 4; total 78, Needs Review empty.

Gate green: validate 0 warnings, selftest 23/23, smoke 15 pages, audit 9 pages.
</commit_message>
<xml_diff>
--- a/EventWatch_Customer_Complaints_2026.xlsx
+++ b/EventWatch_Customer_Complaints_2026.xlsx
@@ -2378,13 +2378,13 @@
                 <formatCode>General</formatCode>
                 <ptCount val="3"/>
                 <pt idx="0">
-                  <v>55</v>
+                  <v>56</v>
                 </pt>
                 <pt idx="1">
-                  <v>32</v>
+                  <v>33</v>
                 </pt>
                 <pt idx="2">
-                  <v>8</v>
+                  <v>6</v>
                 </pt>
               </numCache>
             </numRef>
@@ -6128,7 +6128,7 @@
       </c>
       <c r="J24" s="33" t="inlineStr">
         <is>
-          <t>Captured Late</t>
+          <t>Process Clarification</t>
         </is>
       </c>
       <c r="K24" s="33" t="inlineStr">
@@ -9025,12 +9025,12 @@
       </c>
       <c r="I52" s="33" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>Product</t>
         </is>
       </c>
       <c r="J52" s="33" t="inlineStr">
         <is>
-          <t>WarRoom Creation</t>
+          <t>Source Coverage</t>
         </is>
       </c>
       <c r="K52" s="33" t="inlineStr">
@@ -9084,7 +9084,7 @@
       <c r="X52" s="33" t="n"/>
       <c r="Y52" s="33" t="inlineStr">
         <is>
-          <t>EventWatch Ops - Nitin Rindhe</t>
+          <t>Product &amp; Platform</t>
         </is>
       </c>
       <c r="Z52" s="37" t="n"/>
@@ -14587,12 +14587,12 @@
       </c>
       <c r="I103" s="33" t="inlineStr">
         <is>
-          <t>Process</t>
+          <t>People</t>
         </is>
       </c>
       <c r="J103" s="33" t="inlineStr">
         <is>
-          <t>Captured Late</t>
+          <t>Review</t>
         </is>
       </c>
       <c r="K103" s="33" t="inlineStr">

</xml_diff>

<commit_message>
Set EAO-39 Fix Status to RCA Shared
The owner's choice from the four allowed values, in place of the spec's
"Closed" which the column does not carry. All four Alerting Gap rows now
read RCA Shared.

Reconciliation unchanged: 124 rows, 85 confirmed misses, 4 Alerting Gap.

Gates: validate.py PASS (0 warnings), smoke_app.py PASS, audit_pages.py
PASS.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FHaiZAbQ4hsiftTWXhdhmi
</commit_message>
<xml_diff>
--- a/EventWatch_Customer_Complaints_2026.xlsx
+++ b/EventWatch_Customer_Complaints_2026.xlsx
@@ -1771,10 +1771,10 @@
                   <v>45</v>
                 </pt>
                 <pt idx="1">
-                  <v>36</v>
+                  <v>37</v>
                 </pt>
                 <pt idx="2">
-                  <v>16</v>
+                  <v>15</v>
                 </pt>
                 <pt idx="3">
                   <v>6</v>
@@ -15054,7 +15054,7 @@
       </c>
       <c r="L107" s="33" t="inlineStr">
         <is>
-          <t>Clarification Provided</t>
+          <t>RCA Shared</t>
         </is>
       </c>
       <c r="M107" s="33" t="inlineStr">

</xml_diff>

<commit_message>
Close EAO-51 as RCA Shared
The RCA went to General Mills on 13-Oct-2026 as an attachment on EAO-51.
`Short Term Fix Status` moves off `Pending`; `RCA Details` records that the RCA
was issued and that its text is not in the ticket, rather than paraphrasing a
document nobody can read back.

`Resolution Date` stays blank: the ticket is still open at Approval Requested
with `resolutiondate` null, and a guessed date is worse than none. The
classification is untouched -- People / Review, routed to EventWatch Ops -- and
three of the four articles raised with monitoring are still unaccounted for,
which the RCA text now says.

Dashboard effect is the Fix Status cache only: RCA Shared 37 -> 38, Pending
6 -> 5. No miss count moves.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FHaiZAbQ4hsiftTWXhdhmi
</commit_message>
<xml_diff>
--- a/EventWatch_Customer_Complaints_2026.xlsx
+++ b/EventWatch_Customer_Complaints_2026.xlsx
@@ -1771,13 +1771,13 @@
                   <v>45</v>
                 </pt>
                 <pt idx="1">
-                  <v>37</v>
+                  <v>38</v>
                 </pt>
                 <pt idx="2">
                   <v>15</v>
                 </pt>
                 <pt idx="3">
-                  <v>6</v>
+                  <v>5</v>
                 </pt>
               </numCache>
             </numRef>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="L112" s="33" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>RCA Shared</t>
         </is>
       </c>
       <c r="M112" s="33" t="inlineStr">
@@ -15672,7 +15672,7 @@
       </c>
       <c r="X112" s="33" t="inlineStr">
         <is>
-          <t>Four articles were raised with monitoring. Engineering traced one of them (undercodenews) and found it had been captured by the cyber attack RSS and linked to an existing cluster (cyber_attack_dt_20260915155539357_not.impactful._) which was later marked as not impactful; the other three are not accounted for yet. The owner classifies this as a People issue: the story did reach the portal and the not-impactful call was made by a person, so the failure is the quality of that review rather than the reach of the system. Not a source-coverage gap - the row carried that reading before the investigation reported, and it is corrected here. Under investigation: no agreed RCA yet.</t>
+          <t>Four articles were raised with monitoring. Engineering traced one of them (undercodenews) and found it had been captured by the cyber attack RSS and linked to an existing cluster (cyber_attack_dt_20260915155539357_not.impactful._) which was later marked as not impactful; the other three are not accounted for yet. The owner classifies this as a People issue: the story did reach the portal and the not-impactful call was made by a person, so the failure is the quality of that review rather than the reach of the system. Not a source-coverage gap - the row carried that reading before the investigation reported, and it is corrected here. An RCA was issued to General Mills on 13-Oct-2026 as an attachment on EAO-51. Its text is not in the ticket, so it is not reproduced here. The ticket is still open at Approval Requested, and three of the four articles raised with monitoring are not yet accounted for.</t>
         </is>
       </c>
       <c r="Y112" s="33" t="inlineStr">

</xml_diff>

<commit_message>
Close EAO-51 as RCA Shared (#99)
The RCA went to General Mills on 13-Oct-2026 as an attachment on EAO-51.
`Short Term Fix Status` moves off `Pending`; `RCA Details` records that the RCA
was issued and that its text is not in the ticket, rather than paraphrasing a
document nobody can read back.

`Resolution Date` stays blank: the ticket is still open at Approval Requested
with `resolutiondate` null, and a guessed date is worse than none. The
classification is untouched -- People / Review, routed to EventWatch Ops -- and
three of the four articles raised with monitoring are still unaccounted for,
which the RCA text now says.

Dashboard effect is the Fix Status cache only: RCA Shared 37 -> 38, Pending
6 -> 5. No miss count moves.


Claude-Session: https://claude.ai/code/session_01FHaiZAbQ4hsiftTWXhdhmi

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/EventWatch_Customer_Complaints_2026.xlsx
+++ b/EventWatch_Customer_Complaints_2026.xlsx
@@ -1771,13 +1771,13 @@
                   <v>45</v>
                 </pt>
                 <pt idx="1">
-                  <v>37</v>
+                  <v>38</v>
                 </pt>
                 <pt idx="2">
                   <v>15</v>
                 </pt>
                 <pt idx="3">
-                  <v>6</v>
+                  <v>5</v>
                 </pt>
               </numCache>
             </numRef>
@@ -15622,7 +15622,7 @@
       </c>
       <c r="L112" s="33" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>RCA Shared</t>
         </is>
       </c>
       <c r="M112" s="33" t="inlineStr">
@@ -15672,7 +15672,7 @@
       </c>
       <c r="X112" s="33" t="inlineStr">
         <is>
-          <t>Four articles were raised with monitoring. Engineering traced one of them (undercodenews) and found it had been captured by the cyber attack RSS and linked to an existing cluster (cyber_attack_dt_20260915155539357_not.impactful._) which was later marked as not impactful; the other three are not accounted for yet. The owner classifies this as a People issue: the story did reach the portal and the not-impactful call was made by a person, so the failure is the quality of that review rather than the reach of the system. Not a source-coverage gap - the row carried that reading before the investigation reported, and it is corrected here. Under investigation: no agreed RCA yet.</t>
+          <t>Four articles were raised with monitoring. Engineering traced one of them (undercodenews) and found it had been captured by the cyber attack RSS and linked to an existing cluster (cyber_attack_dt_20260915155539357_not.impactful._) which was later marked as not impactful; the other three are not accounted for yet. The owner classifies this as a People issue: the story did reach the portal and the not-impactful call was made by a person, so the failure is the quality of that review rather than the reach of the system. Not a source-coverage gap - the row carried that reading before the investigation reported, and it is corrected here. An RCA was issued to General Mills on 13-Oct-2026 as an attachment on EAO-51. Its text is not in the ticket, so it is not reproduced here. The ticket is still open at Approval Requested, and three of the four articles raised with monitoring are not yet accounted for.</t>
         </is>
       </c>
       <c r="Y112" s="33" t="inlineStr">

</xml_diff>

<commit_message>
EAO-52: corrective action complete, row leaves Pending
Engineering added the Carlisle keywords to two RSS feeds on 14-Oct-2026,
which closes the investigation, so Short Term Fix Status moves Pending ->
Fixed. Resolution Date stays blank: the ticket carries no resolutiondate.

The row's own Comments now name what is still outstanding, because nothing
automatic looks at a row once it leaves Pending -- the written RCA is in
internal approval with PM and has not gone to General Mills, and the
geofencing and WarRoom-creation questions are unanswered.

Sub-type untouched. Engineering's 'this is a keyword miss' is a proposal,
not a licence to apply, and the row already read Keyword Update.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FHaiZAbQ4hsiftTWXhdhmi
</commit_message>
<xml_diff>
--- a/EventWatch_Customer_Complaints_2026.xlsx
+++ b/EventWatch_Customer_Complaints_2026.xlsx
@@ -1768,7 +1768,7 @@
                 <formatCode>General</formatCode>
                 <ptCount val="4"/>
                 <pt idx="0">
-                  <v>45</v>
+                  <v>46</v>
                 </pt>
                 <pt idx="1">
                   <v>40</v>
@@ -1777,7 +1777,7 @@
                   <v>14</v>
                 </pt>
                 <pt idx="3">
-                  <v>4</v>
+                  <v>3</v>
                 </pt>
               </numCache>
             </numRef>
@@ -16664,7 +16664,7 @@
       </c>
       <c r="L121" s="33" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="M121" s="33" t="inlineStr">
@@ -16679,7 +16679,7 @@
       </c>
       <c r="O121" s="33" t="inlineStr">
         <is>
-          <t>Staged from Jira EAO-52 (Open). General Mills reported that a complete municipal water supply disruption and a citywide do-not-use-water order hit their Carlisle, Iowa flour mill on 30-Sep-2026, temporarily disrupting milling operations and requiring 2,500-gallon water tankers as mitigation, and that no WarRoom notification was generated. The customer confirms the Carlisle facility has been in their CDIF/site data since inception, including site ID, address, city and state, and that news coverage named Carlisle, Iowa explicitly. The ticket asks whether the event was captured by monitoring at all, why it was not associated with the facility if it was, and why no WarRoom followed. Engineering confirmed on 12-Oct-2026 that this is a keyword miss and that the keyword is being added, so the Sub-type is no longer a staging guess; the ticket is still open with PM and the geofencing and WarRoom questions have not been answered separately. Under investigation: no agreed RCA yet.</t>
+          <t>Staged from Jira EAO-52 (Open). General Mills reported that a complete municipal water supply disruption and a citywide do-not-use-water order hit their Carlisle, Iowa flour mill on 30-Sep-2026, temporarily disrupting milling operations and requiring 2,500-gallon water tankers as mitigation, and that no WarRoom notification was generated. The customer confirms the Carlisle facility has been in their CDIF/site data since inception, including site ID, address, city and state, and that news coverage named Carlisle, Iowa explicitly. The ticket asks whether the event was captured by monitoring at all, why it was not associated with the facility if it was, and why no WarRoom followed. Engineering confirmed on 12-Oct-2026 that this is a keyword miss and added the keywords to two RSS feeds on 14-Oct-2026, so the corrective action is complete and the row leaves Pending. STILL OPEN, and nothing automatic will look at this row again: the written RCA was attached on 14-Oct-2026 and is in internal approval with PM, not yet shared with General Mills, so there is no Resolution Date; the geofencing and WarRoom-creation questions the customer raised have not been answered separately. The Sub-type reads Keyword Update on engineering's own wording and awaits the owner's confirmation.</t>
         </is>
       </c>
       <c r="P121" s="33" t="n"/>
@@ -16714,7 +16714,7 @@
       </c>
       <c r="X121" s="33" t="inlineStr">
         <is>
-          <t>Monitoring checked the Not Impacted tab and found no relevant article, then established the cause as a keyword miss: the Carlisle coverage was not matched by the algorithm's keyword set. The keyword is being added. Not a source-coverage gap - the row was staged as one before the investigation reported, and is corrected here.</t>
+          <t>Monitoring checked the Not Impacted tab and found no relevant article, then established the cause as a keyword miss: the Carlisle coverage was not matched by the algorithm's keyword set. Engineering added the keywords to two RSS feeds on 14-Oct-2026. Not a source-coverage gap - the row was staged as one before the investigation reported, and is corrected here. A written RCA was attached to the ticket on 14-Oct-2026 and its text is not readable from Jira.</t>
         </is>
       </c>
       <c r="Y121" s="33" t="inlineStr">

</xml_diff>